<commit_message>
fix(fii-flows): correct FY2026-27 to match its monthly data (-100369, was a bad -143784 source cell); recompute cum tail — cumulative line now internally consistent
</commit_message>
<xml_diff>
--- a/tools/fii-flows/FII_FPI_Historical_Data_India.xlsx
+++ b/tools/fii-flows/FII_FPI_Historical_Data_India.xlsx
@@ -1079,10 +1079,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>-180832</v>
+        <v>-180834</v>
       </c>
       <c r="C35" t="n">
-        <v>25807</v>
+        <v>28143</v>
       </c>
       <c r="D35" t="n">
         <v>-152691</v>
@@ -1098,16 +1098,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>-150195</v>
+        <v>-93810</v>
       </c>
       <c r="C36" t="n">
-        <v>4924</v>
+        <v>-6559</v>
       </c>
       <c r="D36" t="n">
-        <v>-143784</v>
+        <v>-100369</v>
       </c>
       <c r="E36" t="n">
-        <v>1340619</v>
+        <v>1384034</v>
       </c>
     </row>
   </sheetData>
@@ -1550,7 +1550,7 @@
         <v>-166286</v>
       </c>
       <c r="C25" t="n">
-        <v>58348</v>
+        <v>62236</v>
       </c>
       <c r="D25" t="n">
         <v>-104050</v>
@@ -1567,7 +1567,7 @@
         <v>-224932</v>
       </c>
       <c r="C26" t="n">
-        <v>8266</v>
+        <v>7391</v>
       </c>
       <c r="D26" t="n">
         <v>-217541</v>

</xml_diff>